<commit_message>
Add Chambers Point as a fifth shop with its own day export and per-shop price sync
Chambers Point now has a shop choice, its own price-list sheet, an admin
smoke test suite, and a dedicated daily download kept out of the combined
All Shops workbook. Add sync_shop_prices to load per-shop price overrides
from each "price list - <Shop>.xlsx" sheet.

🤖 Generated with Codebuff 🤖

Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/price list - Emirates.xlsx
+++ b/price list - Emirates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D109"/>
+  <dimension ref="A1:D110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -873,11 +873,11 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Chrome Vodka</t>
+          <t>Chrome brandy</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>208</v>
+        <v>225</v>
       </c>
       <c r="C26" t="n">
         <v>300</v>
@@ -895,32 +895,32 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>610</v>
+        <v>208</v>
       </c>
       <c r="C27" t="n">
-        <v>1000</v>
+        <v>300</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>750ml</t>
+          <t>250ml</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Chrome Gin</t>
+          <t>Chrome Vodka</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>210</v>
+        <v>610</v>
       </c>
       <c r="C28" t="n">
-        <v>300</v>
+        <v>1000</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>250ml</t>
+          <t>750ml</t>
         </is>
       </c>
     </row>
@@ -931,28 +931,28 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>610</v>
+        <v>210</v>
       </c>
       <c r="C29" t="n">
-        <v>1000</v>
+        <v>300</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>750ml</t>
+          <t>250ml</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Imperial Blue</t>
+          <t>Chrome Gin</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0</v>
+        <v>610</v>
       </c>
       <c r="C30" t="n">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -963,18 +963,18 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Origin</t>
+          <t>Imperial Blue</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>232</v>
+        <v>0</v>
       </c>
       <c r="C31" t="n">
-        <v>300</v>
+        <v>1600</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>250ml</t>
+          <t>750ml</t>
         </is>
       </c>
     </row>
@@ -985,21 +985,21 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0</v>
+        <v>232</v>
       </c>
       <c r="C32" t="n">
-        <v>1100</v>
+        <v>300</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>750ml</t>
+          <t>250ml</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>4th street</t>
+          <t>Origin</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1017,14 +1017,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>jameson 1l</t>
+          <t>4th street</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>3000</v>
+        <v>1100</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1035,14 +1035,14 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Jameson 750ml</t>
+          <t>jameson 1l</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1053,14 +1053,14 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>William Lawsons</t>
+          <t>Jameson 750ml</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>0</v>
       </c>
       <c r="C36" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1071,18 +1071,18 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>viceroy</t>
+          <t>William Lawsons</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>395</v>
+        <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>550</v>
+        <v>2000</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>250ml</t>
+          <t>750ml</t>
         </is>
       </c>
     </row>
@@ -1093,32 +1093,32 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1200</v>
+        <v>395</v>
       </c>
       <c r="C38" t="n">
-        <v>1500</v>
+        <v>550</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>750ml</t>
+          <t>250ml</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Black&amp;white</t>
+          <t>viceroy</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="C39" t="n">
-        <v>1100</v>
+        <v>1500</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>350ml</t>
+          <t>750ml</t>
         </is>
       </c>
     </row>
@@ -1129,32 +1129,32 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="C40" t="n">
-        <v>1500</v>
+        <v>1100</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>750ml</t>
+          <t>350ml</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Gilbeys</t>
+          <t>Black&amp;white</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>416</v>
+        <v>1000</v>
       </c>
       <c r="C41" t="n">
-        <v>550</v>
+        <v>1500</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>250ml</t>
+          <t>750ml</t>
         </is>
       </c>
     </row>
@@ -1165,14 +1165,14 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>580</v>
+        <v>416</v>
       </c>
       <c r="C42" t="n">
-        <v>850</v>
+        <v>550</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>350ml</t>
+          <t>250ml</t>
         </is>
       </c>
     </row>
@@ -1186,29 +1186,29 @@
         <v>580</v>
       </c>
       <c r="C43" t="n">
-        <v>1500</v>
+        <v>850</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>750ml</t>
+          <t>350ml</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Captain Morgan</t>
+          <t>Gilbeys</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>334</v>
+        <v>580</v>
       </c>
       <c r="C44" t="n">
-        <v>400</v>
+        <v>1500</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>250ml</t>
+          <t>750ml</t>
         </is>
       </c>
     </row>
@@ -1219,32 +1219,32 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>910</v>
+        <v>334</v>
       </c>
       <c r="C45" t="n">
-        <v>1200</v>
+        <v>400</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>750ml</t>
+          <t>250ml</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>County</t>
+          <t>Captain Morgan</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>231</v>
+        <v>910</v>
       </c>
       <c r="C46" t="n">
-        <v>300</v>
+        <v>1200</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>250ml</t>
+          <t>750ml</t>
         </is>
       </c>
     </row>
@@ -1255,32 +1255,32 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>670</v>
+        <v>231</v>
       </c>
       <c r="C47" t="n">
-        <v>1000</v>
+        <v>300</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>750ml</t>
+          <t>250ml</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Smirnoff</t>
+          <t>County</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>350</v>
+        <v>670</v>
       </c>
       <c r="C48" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>250ml</t>
+          <t>750ml</t>
         </is>
       </c>
     </row>
@@ -1291,14 +1291,14 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0</v>
+        <v>350</v>
       </c>
       <c r="C49" t="n">
-        <v>850</v>
+        <v>500</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>350ml</t>
+          <t>250ml</t>
         </is>
       </c>
     </row>
@@ -1312,29 +1312,29 @@
         <v>0</v>
       </c>
       <c r="C50" t="n">
-        <v>1400</v>
+        <v>850</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>750ml</t>
+          <t>350ml</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Kibao</t>
+          <t>Smirnoff</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>225</v>
+        <v>0</v>
       </c>
       <c r="C51" t="n">
-        <v>300</v>
+        <v>1400</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>250ml</t>
+          <t>750ml</t>
         </is>
       </c>
     </row>
@@ -1345,14 +1345,14 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>320</v>
+        <v>225</v>
       </c>
       <c r="C52" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>350ml</t>
+          <t>250ml</t>
         </is>
       </c>
     </row>
@@ -1363,32 +1363,32 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="C53" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>750ml</t>
+          <t>350ml</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>General Meakings</t>
+          <t>Kibao</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="C54" t="n">
-        <v>300</v>
+        <v>1000</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>250ml</t>
+          <t>750ml</t>
         </is>
       </c>
     </row>
@@ -1399,28 +1399,28 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>600</v>
+        <v>210</v>
       </c>
       <c r="C55" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>750ml</t>
+          <t>250ml</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Amarula 1ltr</t>
+          <t>General Meakings</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="C56" t="n">
-        <v>3000</v>
+        <v>900</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -1431,14 +1431,14 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Amarula 750</t>
+          <t>Amarula 1ltr</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>0</v>
       </c>
       <c r="C57" t="n">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -1449,14 +1449,14 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Best Gin</t>
+          <t>Amarula 750</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>0</v>
       </c>
       <c r="C58" t="n">
-        <v>950</v>
+        <v>2500</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1467,14 +1467,14 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Best Whisky</t>
+          <t>Best Gin</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>0</v>
       </c>
       <c r="C59" t="n">
-        <v>1200</v>
+        <v>950</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -1485,14 +1485,14 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Red label 750</t>
+          <t>Best Whisky</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>0</v>
       </c>
       <c r="C60" t="n">
-        <v>2200</v>
+        <v>1200</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1503,14 +1503,14 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Red label 375ml</t>
+          <t>Red label 750</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>0</v>
       </c>
       <c r="C61" t="n">
-        <v>1300</v>
+        <v>2200</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -1521,14 +1521,14 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Red Label 1 ltr</t>
+          <t>Red label 375ml</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>0</v>
       </c>
       <c r="C62" t="n">
-        <v>2600</v>
+        <v>1300</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -1539,14 +1539,14 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Black Label 375ml</t>
+          <t>Red Label 1 ltr</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>0</v>
       </c>
       <c r="C63" t="n">
-        <v>2250</v>
+        <v>2600</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -1557,14 +1557,14 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Black Label 750ml</t>
+          <t>Black Label 375ml</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>0</v>
       </c>
       <c r="C64" t="n">
-        <v>3500</v>
+        <v>2250</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -1575,14 +1575,14 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Black Label 1ltr</t>
+          <t>Black Label 750ml</t>
         </is>
       </c>
       <c r="B65" t="n">
         <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>4000</v>
+        <v>3500</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -1593,14 +1593,14 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Drostody hol</t>
+          <t>Black Label 1ltr</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>0</v>
       </c>
       <c r="C66" t="n">
-        <v>1000</v>
+        <v>4000</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -1611,18 +1611,18 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Richot</t>
+          <t>Drostody hol</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>358</v>
+        <v>0</v>
       </c>
       <c r="C67" t="n">
-        <v>550</v>
+        <v>1000</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>250ml</t>
+          <t>750ml</t>
         </is>
       </c>
     </row>
@@ -1633,14 +1633,14 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>0</v>
+        <v>358</v>
       </c>
       <c r="C68" t="n">
-        <v>800</v>
+        <v>550</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>350ml</t>
+          <t>250ml</t>
         </is>
       </c>
     </row>
@@ -1654,25 +1654,25 @@
         <v>0</v>
       </c>
       <c r="C69" t="n">
-        <v>1500</v>
+        <v>800</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>750ml</t>
+          <t>350ml</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>VAT 69</t>
+          <t>Richot</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>0</v>
       </c>
       <c r="C70" t="n">
-        <v>1800</v>
+        <v>1500</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -1683,25 +1683,25 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Guarana</t>
+          <t>VAT 69</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>175</v>
+        <v>0</v>
       </c>
       <c r="C71" t="n">
-        <v>250</v>
+        <v>1800</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>cans</t>
+          <t>750ml</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Guarana Black</t>
+          <t>Guarana</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1719,14 +1719,14 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Tusker</t>
+          <t>Guarana Black</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>198</v>
+        <v>175</v>
       </c>
       <c r="C73" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -1737,11 +1737,11 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Tusker Malt</t>
+          <t>Tusker</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C74" t="n">
         <v>300</v>
@@ -1755,7 +1755,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Tusker Lite</t>
+          <t>Tusker Malt</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1773,11 +1773,11 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Snapp</t>
+          <t>Tusker Lite</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="C76" t="n">
         <v>300</v>
@@ -1791,11 +1791,11 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>pineapple Punch</t>
+          <t>Snapp</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>175</v>
+        <v>0</v>
       </c>
       <c r="C77" t="n">
         <v>300</v>
@@ -1809,11 +1809,11 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Faxe</t>
+          <t>pineapple Punch</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0</v>
+        <v>175</v>
       </c>
       <c r="C78" t="n">
         <v>300</v>
@@ -1827,14 +1827,14 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Redbull</t>
+          <t>Faxe</t>
         </is>
       </c>
       <c r="B79" t="n">
         <v>0</v>
       </c>
       <c r="C79" t="n">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -1845,14 +1845,14 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Delmonte</t>
+          <t>Redbull</t>
         </is>
       </c>
       <c r="B80" t="n">
         <v>0</v>
       </c>
       <c r="C80" t="n">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -1863,14 +1863,14 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Balozi</t>
+          <t>Delmonte</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>245</v>
+        <v>0</v>
       </c>
       <c r="C81" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -1881,14 +1881,14 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Balozi Bottle</t>
+          <t>Balozi</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>169</v>
+        <v>245</v>
       </c>
       <c r="C82" t="n">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -1899,14 +1899,14 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Whitecup</t>
+          <t>Balozi Bottle</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>215</v>
+        <v>169</v>
       </c>
       <c r="C83" t="n">
-        <v>300</v>
+        <v>250</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -1917,14 +1917,14 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Caprice</t>
+          <t>Whitecup</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>600</v>
+        <v>215</v>
       </c>
       <c r="C84" t="n">
-        <v>800</v>
+        <v>300</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -1935,14 +1935,14 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Pilsner Bottle</t>
+          <t>Caprice</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="C85" t="n">
-        <v>270</v>
+        <v>800</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -1953,14 +1953,14 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Heineken</t>
+          <t>Pilsner Bottle</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>169</v>
+        <v>200</v>
       </c>
       <c r="C86" t="n">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -1971,47 +1971,47 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Tusker Bottle</t>
+          <t>Heineken</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>198</v>
+        <v>169</v>
       </c>
       <c r="C87" t="n">
-        <v>270</v>
+        <v>300</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Bottle</t>
+          <t>cans</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Guiness</t>
+          <t>Tusker Bottle</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>150</v>
+        <v>198</v>
       </c>
       <c r="C88" t="n">
         <v>270</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>cans</t>
+          <t>Bottle</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Guiness Bottle</t>
+          <t>Guiness</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>204</v>
+        <v>150</v>
       </c>
       <c r="C89" t="n">
         <v>270</v>
@@ -2025,11 +2025,11 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Tusker cider</t>
+          <t>Guiness Bottle</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>234</v>
+        <v>204</v>
       </c>
       <c r="C90" t="n">
         <v>270</v>
@@ -2043,11 +2043,11 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Pilsner</t>
+          <t>Tusker cider</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>195</v>
+        <v>234</v>
       </c>
       <c r="C91" t="n">
         <v>270</v>
@@ -2061,7 +2061,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>White Cup Bottle</t>
+          <t>Pilsner</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -2072,21 +2072,21 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>soda</t>
+          <t>cans</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Kingfisher</t>
+          <t>White Cup Bottle</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>0</v>
+        <v>195</v>
       </c>
       <c r="C93" t="n">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -2097,14 +2097,14 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Soda 500ml</t>
+          <t>Kingfisher</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="C94" t="n">
-        <v>80</v>
+        <v>300</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2115,14 +2115,14 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Soda 350ml</t>
+          <t>Soda 500ml</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>41</v>
+        <v>63</v>
       </c>
       <c r="C95" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -2133,14 +2133,14 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Soda 300ml</t>
+          <t>Soda 350ml</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C96" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -2151,14 +2151,14 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Soda 200ml</t>
+          <t>Soda 300ml</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C97" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -2169,14 +2169,14 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Soda 1.25ltrs</t>
+          <t>Soda 200ml</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="C98" t="n">
-        <v>180</v>
+        <v>30</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -2187,14 +2187,14 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>soda 1ltr</t>
+          <t>Soda 1.25ltrs</t>
         </is>
       </c>
       <c r="B99" t="n">
         <v>0</v>
       </c>
       <c r="C99" t="n">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -2205,14 +2205,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Soda 2ltrs</t>
+          <t>soda 1ltr</t>
         </is>
       </c>
       <c r="B100" t="n">
         <v>0</v>
       </c>
       <c r="C100" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -2223,14 +2223,14 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>mInutemaid Small</t>
+          <t>Soda 2ltrs</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="C101" t="n">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -2241,14 +2241,14 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>mInutemaid Big</t>
+          <t>mInutemaid Small</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="C102" t="n">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -2259,14 +2259,14 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Dasani Small</t>
+          <t>mInutemaid Big</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="C103" t="n">
-        <v>50</v>
+        <v>160</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -2277,14 +2277,14 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Dasani Big</t>
+          <t>Dasani Small</t>
         </is>
       </c>
       <c r="B104" t="n">
+        <v>33</v>
+      </c>
+      <c r="C104" t="n">
         <v>50</v>
-      </c>
-      <c r="C104" t="n">
-        <v>100</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -2295,14 +2295,14 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Lemonade</t>
+          <t>Dasani Big</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C105" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -2313,14 +2313,14 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>predator</t>
+          <t>Lemonade</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C106" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -2331,14 +2331,14 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Kiss</t>
+          <t>predator</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="C107" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -2349,14 +2349,14 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Glacier Small</t>
+          <t>Kiss</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="C108" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -2367,16 +2367,34 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
+          <t>Glacier Small</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>20</v>
+      </c>
+      <c r="C109" t="n">
+        <v>30</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>soda</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
           <t>Glacier Big</t>
         </is>
       </c>
-      <c r="B109" t="n">
+      <c r="B110" t="n">
         <v>25</v>
       </c>
-      <c r="C109" t="n">
+      <c r="C110" t="n">
         <v>50</v>
       </c>
-      <c r="D109" t="inlineStr">
+      <c r="D110" t="inlineStr">
         <is>
           <t>soda</t>
         </is>

</xml_diff>